<commit_message>
Changed module swaps report to: - Formatting dates properly - Removed decimals - Preventing duplicated data
</commit_message>
<xml_diff>
--- a/api/templates/module_swaps/uk.xlsx
+++ b/api/templates/module_swaps/uk.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26501"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\module_swaps\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\nsabaj\Repositories\aspect\api\templates\module_swaps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E78231E-A2E4-413D-BA4A-A157B1A34906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDB5C1B6-A40D-4813-8DE5-F2998D3B2CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Заміна модулів" sheetId="1" r:id="rId1"/>
@@ -223,7 +223,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -241,9 +241,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -257,11 +254,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -663,171 +676,171 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="41.109375" customWidth="1"/>
-    <col min="2" max="2" width="24.21875" customWidth="1"/>
-    <col min="3" max="3" width="26.33203125" customWidth="1"/>
-    <col min="4" max="4" width="24.21875" customWidth="1"/>
-    <col min="5" max="5" width="15.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="23.109375" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="41.1328125" customWidth="1"/>
+    <col min="2" max="2" width="24.19921875" style="21" customWidth="1"/>
+    <col min="3" max="3" width="26.33203125" style="21" customWidth="1"/>
+    <col min="4" max="4" width="24.19921875" style="26" customWidth="1"/>
+    <col min="5" max="5" width="15.86328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="23.1328125" customWidth="1"/>
+    <col min="7" max="7" width="15.86328125" style="1" customWidth="1"/>
     <col min="8" max="8" width="28" customWidth="1"/>
-    <col min="9" max="9" width="18.5546875" customWidth="1"/>
+    <col min="9" max="9" width="18.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.65">
       <c r="A1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="22"/>
       <c r="E1" s="3"/>
       <c r="F1" s="2"/>
       <c r="G1" s="3"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
     </row>
-    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="6"/>
       <c r="F2" s="5"/>
       <c r="G2" s="6"/>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
     </row>
-    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="23"/>
       <c r="E3" s="6"/>
       <c r="F3" s="5"/>
       <c r="G3" s="6"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
     </row>
-    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="23"/>
       <c r="E4" s="6"/>
       <c r="F4" s="5"/>
       <c r="G4" s="6"/>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
     </row>
-    <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="23"/>
       <c r="E5" s="6"/>
       <c r="F5" s="5"/>
       <c r="G5" s="6"/>
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
     </row>
-    <row r="6" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A6" s="4"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="23"/>
       <c r="E6" s="6"/>
       <c r="F6" s="5"/>
       <c r="G6" s="6"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
     </row>
-    <row r="7" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A7" s="8" t="str">
         <f>"Відсоток заміни модулів в рамках SLA: "&amp;TEXT(COUNTIF(D10:D10002,"&lt;=8")/COUNTIF(D10:D10002,"&lt;&gt;"),"0%")</f>
         <v>Відсоток заміни модулів в рамках SLA: 0%</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="23"/>
       <c r="E7" s="6"/>
       <c r="F7" s="5"/>
       <c r="G7" s="6"/>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
     </row>
-    <row r="8" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:9" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="23"/>
       <c r="E8" s="6"/>
       <c r="F8" s="5"/>
       <c r="G8" s="6"/>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
     </row>
-    <row r="9" spans="1:9" ht="31.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="11" t="s">
+    <row r="9" spans="1:9" ht="31.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A9" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="G9" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="14" t="s">
+    <row r="10" spans="1:9" ht="15.75" x14ac:dyDescent="0.5">
+      <c r="A10" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="F10" s="16" t="s">
+      <c r="F10" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="G10" s="14" t="s">
+      <c r="G10" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="H10" s="17" t="s">
+      <c r="H10" s="15" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>